<commit_message>
feat: ALM engine deep improvement — 4-wave implementation
Wave A (quick wins):
- EVE convexity as first-class engine output (effective duration + convexity)
- Sensitivity explain rewrite with per-deal waterfall reconciliation
- Data quality: rate bounds, duplicate deals, maturity/sign consistency checks

Wave B (core improvements):
- Rate-dependent CPR wired into EVE scenarios via nominal_adjuster callback
- NMD beta/decay stress under large shocks (>200bp threshold)
- Budget variance waterfall decomposition (volume/rate/new/matured effects)

Wave C (strategic features):
- Multi-tenor hedge optimizer (1Y-10Y) with KRD-based and curve-aware selection
- FTP 3-way ALM margin decomposition (duration/credit/liquidity)

Wave D (advanced):
- Dynamic balance sheet simulation with production plan reinvestment
- Production plan Excel parser and auto-discovery in render pipeline

All 608 tests pass. Fully backward compatible.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/ideal_input/deals.xlsx
+++ b/tests/fixtures/ideal_input/deals.xlsx
@@ -509,37 +509,37 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>pay_receive</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>indexation</t>
+          <t>notional</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>instrument_type</t>
+          <t>last_fixing_date</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>pay_receive</t>
+          <t>next_fixing_date</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>notional</t>
+          <t>hedge_type</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>last_fixing_date</t>
+          <t>ias_standard</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>next_fixing_date</t>
+          <t>designation_date</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,11 @@
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>STRAT_CHF_001</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>CC</t>
@@ -612,21 +616,25 @@
           <t>THCCBFIGE</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Act/360</t>
-        </is>
-      </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Deposit</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>cash_flow</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>IFRS9</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2025-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -697,17 +705,9 @@
           <t>BKCCBFIGE</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Act/360</t>
-        </is>
-      </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Deposit</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
@@ -771,7 +771,11 @@
           <t>2027-06-12</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>STRAT_CHF_002</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr">
         <is>
           <t>CC</t>
@@ -782,21 +786,25 @@
           <t>THCCBFIGE</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Act/360</t>
-        </is>
-      </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Loan</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>fair_value</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>IAS39</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -871,17 +879,9 @@
           <t>WCCCBFIGE</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Act/360</t>
-        </is>
-      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Loan</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
@@ -956,17 +956,9 @@
           <t>THCCHFIGE</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>30/360</t>
-        </is>
-      </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Bond</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
@@ -1030,7 +1022,11 @@
           <t>2030-06-17</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>STRAT_EUR_001</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>CC</t>
@@ -1041,21 +1037,25 @@
           <t>BKCCBFIGE</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>30/360</t>
-        </is>
-      </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Bond</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>cash_flow</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>IFRS9</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1126,17 +1126,9 @@
           <t>CLI-MT-CIB</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>Act/360</t>
-        </is>
-      </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>FX Swap</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
@@ -1211,17 +1203,9 @@
           <t>THCCBFIGE</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Act/365</t>
-        </is>
-      </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Deposit</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
@@ -1285,11 +1269,7 @@
           <t>2028-02-03</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>STRAT_001</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
           <t>CC</t>
@@ -1300,17 +1280,9 @@
           <t>THCCBFIGE</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Act/360</t>
-        </is>
-      </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Deposit</t>
-        </is>
-      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
@@ -1385,17 +1357,9 @@
           <t>THCCBFIGE</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Act/360</t>
-        </is>
-      </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Deposit</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -1463,7 +1427,11 @@
           <t>2030-03-17</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>STRAT_CHF_001</t>
+        </is>
+      </c>
       <c r="Q12" t="inlineStr">
         <is>
           <t>CC</t>
@@ -1476,31 +1444,35 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Act/360</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr"/>
+          <t>PAY</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>100000000</v>
+      </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>IRS</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>PAY</t>
-        </is>
-      </c>
-      <c r="W12" t="n">
-        <v>100000000</v>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>cash_flow</t>
+        </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>IFRS9</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2025-06-15</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1538,11 @@
           <t>2029-11-03</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>STRAT_CHF_002</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>CC</t>
@@ -1579,31 +1555,35 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Act/360</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr"/>
+          <t>RECEIVE</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>75000000</v>
+      </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>IRS</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>RECEIVE</t>
-        </is>
-      </c>
-      <c r="W13" t="n">
-        <v>75000000</v>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>fair_value</t>
+        </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>IAS39</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2025-01-20</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1649,11 @@
           <t>2028-06-03</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>STRAT_EUR_001</t>
+        </is>
+      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>CC</t>
@@ -1682,31 +1666,35 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Act/360</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr"/>
+          <t>PAY</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>50000000</v>
+      </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>IRS</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>PAY</t>
-        </is>
-      </c>
-      <c r="W14" t="n">
-        <v>50000000</v>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>cash_flow</t>
+        </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>IFRS9</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2025-09-01</t>
         </is>
       </c>
     </row>

</xml_diff>